<commit_message>
Updated for 11 August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/Python Data set/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2A1BC998-7EF3-41CF-AB82-D8B4E43F459D}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA44DFFF-ECFC-4D3F-B368-E6EBAB508CAC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1045,21 +1045,31 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9"/>
+      <c r="A7" s="8">
+        <v>46245</v>
+      </c>
+      <c r="B7" s="9">
+        <v>390</v>
+      </c>
+      <c r="C7" s="9">
+        <v>60</v>
+      </c>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
-      <c r="F7" s="9"/>
-      <c r="G7" s="9"/>
+      <c r="F7" s="9">
+        <v>250</v>
+      </c>
+      <c r="G7" s="9">
+        <v>5</v>
+      </c>
       <c r="H7" s="9"/>
-      <c r="I7" s="10" t="str">
+      <c r="I7" s="10">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J7" s="10" t="str">
+        <v>700</v>
+      </c>
+      <c r="J7" s="10">
         <f t="shared" si="1"/>
-        <v/>
+        <v>740</v>
       </c>
       <c r="K7" s="11"/>
       <c r="L7" s="11"/>

</xml_diff>

<commit_message>
Updated ver2.0 for 11 Aug
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AA44DFFF-ECFC-4D3F-B368-E6EBAB508CAC}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{402187DD-1D25-42C4-8CD7-08912443E41F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -214,7 +214,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,6 +308,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -356,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -402,6 +417,21 @@
     <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="15" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -498,6 +528,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1044,37 +1078,37 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A7" s="8">
+    <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="23">
         <v>46245</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="24">
         <v>390</v>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="24">
         <v>60</v>
       </c>
-      <c r="D7" s="9"/>
-      <c r="E7" s="9"/>
-      <c r="F7" s="9">
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+      <c r="F7" s="24">
         <v>250</v>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="24">
         <v>5</v>
       </c>
-      <c r="H7" s="9"/>
-      <c r="I7" s="10">
+      <c r="H7" s="24"/>
+      <c r="I7" s="25">
         <f t="shared" si="0"/>
         <v>700</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="25">
         <f t="shared" si="1"/>
         <v>740</v>
       </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="12"/>
+      <c r="K7" s="26"/>
+      <c r="L7" s="26"/>
+      <c r="M7" s="26"/>
+      <c r="N7" s="27"/>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>

</xml_diff>

<commit_message>
Full Update for 11th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{402187DD-1D25-42C4-8CD7-08912443E41F}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F34A6B55-9EE1-4503-8CD2-94A0534661F1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -205,6 +205,15 @@
   </si>
   <si>
     <t>I was enthusiastic about the test but felt very tired due to taking stairs.</t>
+  </si>
+  <si>
+    <t>Neutral</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Today I did some coding in cpp &amp; read some more about DBMS.</t>
   </si>
 </sst>
 </file>
@@ -412,11 +421,6 @@
     <xf numFmtId="0" fontId="13" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -432,6 +436,11 @@
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -921,72 +930,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="24" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B2" s="20" t="s">
+      <c r="B2" s="25" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="22">
+      <c r="F2" s="27">
         <v>12601870</v>
       </c>
-      <c r="G2" s="22"/>
+      <c r="G2" s="27"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="25" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="21"/>
-      <c r="D3" s="21"/>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
       <c r="E3" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="25" t="s">
         <v>53</v>
       </c>
-      <c r="G3" s="21"/>
+      <c r="G3" s="26"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="18"/>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
+      <c r="A4" s="23"/>
+      <c r="B4" s="23"/>
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="23"/>
+      <c r="G4" s="23"/>
+      <c r="H4" s="23"/>
+      <c r="I4" s="23"/>
+      <c r="J4" s="23"/>
+      <c r="K4" s="23"/>
+      <c r="L4" s="23"/>
+      <c r="M4" s="23"/>
+      <c r="N4" s="23"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -1078,37 +1087,51 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A7" s="23">
+    <row r="7" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="18">
         <v>46245</v>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="19">
         <v>390</v>
       </c>
-      <c r="C7" s="24">
+      <c r="C7" s="19">
         <v>60</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24"/>
-      <c r="F7" s="24">
+      <c r="D7" s="19">
+        <v>172</v>
+      </c>
+      <c r="E7" s="19">
+        <v>60</v>
+      </c>
+      <c r="F7" s="19">
         <v>250</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="19">
         <v>5</v>
       </c>
-      <c r="H7" s="24"/>
-      <c r="I7" s="25">
+      <c r="H7" s="19">
+        <v>180</v>
+      </c>
+      <c r="I7" s="20">
         <f t="shared" si="0"/>
-        <v>700</v>
-      </c>
-      <c r="J7" s="25">
+        <v>1112</v>
+      </c>
+      <c r="J7" s="20">
         <f t="shared" si="1"/>
-        <v>740</v>
-      </c>
-      <c r="K7" s="26"/>
-      <c r="L7" s="26"/>
-      <c r="M7" s="26"/>
-      <c r="N7" s="27"/>
+        <v>328</v>
+      </c>
+      <c r="K7" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="L7" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="M7" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N7" s="22" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>

</xml_diff>

<commit_message>
Updated for 12th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F34A6B55-9EE1-4503-8CD2-94A0534661F1}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B17BD4C-728F-4475-AE55-2813259AD57D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -214,6 +214,9 @@
   </si>
   <si>
     <t>Today I did some coding in cpp &amp; read some more about DBMS.</t>
+  </si>
+  <si>
+    <t>Today was the most hectic day coz Today there were 8 classes back to back &amp; it was a proper body as well as mental exhaustion.</t>
   </si>
 </sst>
 </file>
@@ -1133,27 +1136,51 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="8"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="9"/>
-      <c r="G8" s="9"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10" t="str">
+    <row r="8" spans="1:14" ht="78" x14ac:dyDescent="0.3">
+      <c r="A8" s="18">
+        <v>46246</v>
+      </c>
+      <c r="B8" s="19">
+        <v>330</v>
+      </c>
+      <c r="C8" s="19">
+        <v>26</v>
+      </c>
+      <c r="D8" s="19">
+        <v>90</v>
+      </c>
+      <c r="E8" s="19">
+        <v>45</v>
+      </c>
+      <c r="F8" s="19">
+        <v>400</v>
+      </c>
+      <c r="G8" s="19">
+        <v>8</v>
+      </c>
+      <c r="H8" s="19">
+        <v>175</v>
+      </c>
+      <c r="I8" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="10" t="str">
+        <v>1066</v>
+      </c>
+      <c r="J8" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="12"/>
+        <v>374</v>
+      </c>
+      <c r="K8" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="L8" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M8" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N8" s="22" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="8"/>

</xml_diff>

<commit_message>
Updated for August 13th
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6B17BD4C-728F-4475-AE55-2813259AD57D}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75E51FEB-2B17-4D7E-B4D5-AE046D91AB7B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="63">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -217,6 +217,15 @@
   </si>
   <si>
     <t>Today was the most hectic day coz Today there were 8 classes back to back &amp; it was a proper body as well as mental exhaustion.</t>
+  </si>
+  <si>
+    <t>Stressed</t>
+  </si>
+  <si>
+    <t>Unsatisfied</t>
+  </si>
+  <si>
+    <t>Back to back 7 ~ 8 classes did a heavy tole on my body, After coming back from the classes I just slept for 1 hour straight then ate some food then do some home work &amp; now will go to sleep again</t>
   </si>
 </sst>
 </file>
@@ -1182,71 +1191,95 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="9"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9"/>
-      <c r="I9" s="10" t="str">
+    <row r="9" spans="1:14" ht="124.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="18">
+        <v>46247</v>
+      </c>
+      <c r="B9" s="19">
+        <v>410</v>
+      </c>
+      <c r="C9" s="19">
+        <v>45</v>
+      </c>
+      <c r="D9" s="19">
+        <v>30</v>
+      </c>
+      <c r="E9" s="19">
+        <v>0</v>
+      </c>
+      <c r="F9" s="19">
+        <v>350</v>
+      </c>
+      <c r="G9" s="19">
+        <v>7</v>
+      </c>
+      <c r="H9" s="19">
+        <v>65</v>
+      </c>
+      <c r="I9" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J9" s="10" t="str">
+        <v>900</v>
+      </c>
+      <c r="J9" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="12"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A10" s="8"/>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="9"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="10" t="str">
+        <v>540</v>
+      </c>
+      <c r="K9" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="L9" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M9" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N9" s="22" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A10" s="18"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="20" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J10" s="10" t="str">
+      <c r="J10" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="12"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A11" s="8"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="10" t="str">
+      <c r="K10" s="21"/>
+      <c r="L10" s="21"/>
+      <c r="M10" s="21"/>
+      <c r="N10" s="22"/>
+    </row>
+    <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="18"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="20" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="J11" s="10" t="str">
+      <c r="J11" s="20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="12"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="22"/>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>

</xml_diff>

<commit_message>
Updated to 14th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75E51FEB-2B17-4D7E-B4D5-AE046D91AB7B}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0ACEC82-22BC-4186-A3A4-06D4115BE2E0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="66">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -226,6 +226,15 @@
   </si>
   <si>
     <t>Back to back 7 ~ 8 classes did a heavy tole on my body, After coming back from the classes I just slept for 1 hour straight then ate some food then do some home work &amp; now will go to sleep again</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Today was the good Day as there were only 3 classes. My body got enough rest &amp; I was able to study in peace.</t>
   </si>
 </sst>
 </file>
@@ -1237,27 +1246,51 @@
         <v>62</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A10" s="18"/>
-      <c r="B10" s="19"/>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="E10" s="19"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="20" t="str">
+    <row r="10" spans="1:14" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A10" s="18">
+        <v>46248</v>
+      </c>
+      <c r="B10" s="19">
+        <v>450</v>
+      </c>
+      <c r="C10" s="19">
+        <v>30</v>
+      </c>
+      <c r="D10" s="19">
+        <v>240</v>
+      </c>
+      <c r="E10" s="19">
+        <v>150</v>
+      </c>
+      <c r="F10" s="19">
+        <v>150</v>
+      </c>
+      <c r="G10" s="19">
+        <v>3</v>
+      </c>
+      <c r="H10" s="19">
+        <v>300</v>
+      </c>
+      <c r="I10" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J10" s="20" t="str">
+        <v>1320</v>
+      </c>
+      <c r="J10" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="21"/>
-      <c r="N10" s="22"/>
+        <v>120</v>
+      </c>
+      <c r="K10" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L10" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N10" s="22" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="18"/>

</xml_diff>

<commit_message>
Updated to 15th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0ACEC82-22BC-4186-A3A4-06D4115BE2E0}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D3A7C95-0295-4D28-A4EB-7D1D2C77FD9C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -235,6 +235,9 @@
   </si>
   <si>
     <t>Today was the good Day as there were only 3 classes. My body got enough rest &amp; I was able to study in peace.</t>
+  </si>
+  <si>
+    <t>Today was THE Independence day &amp; it was the much awaited Holiday, My body is now fully recharged. &amp; I enjoyed all the functions.</t>
   </si>
 </sst>
 </file>
@@ -1292,27 +1295,51 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="18"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="20" t="str">
+    <row r="11" spans="1:14" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A11" s="18">
+        <v>46249</v>
+      </c>
+      <c r="B11" s="19">
+        <v>540</v>
+      </c>
+      <c r="C11" s="19">
+        <v>45</v>
+      </c>
+      <c r="D11" s="19">
+        <v>0</v>
+      </c>
+      <c r="E11" s="19">
+        <v>0</v>
+      </c>
+      <c r="F11" s="19">
+        <v>0</v>
+      </c>
+      <c r="G11" s="19">
+        <v>0</v>
+      </c>
+      <c r="H11" s="19">
+        <v>600</v>
+      </c>
+      <c r="I11" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="20" t="str">
+        <v>1185</v>
+      </c>
+      <c r="J11" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K11" s="21"/>
-      <c r="L11" s="21"/>
-      <c r="M11" s="21"/>
-      <c r="N11" s="22"/>
+        <v>255</v>
+      </c>
+      <c r="K11" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L11" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M11" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N11" s="22" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="8"/>

</xml_diff>

<commit_message>
Updated for 19 August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7F67C9D-0527-4418-9C1C-7634F86CE88F}"/>
+  <xr:revisionPtr revIDLastSave="139" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66EFFD25-626B-401C-9793-6B80229D6872}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -253,6 +253,9 @@
   </si>
   <si>
     <t>Today I have fever &amp; severe body pain, I think it's because of viral. That's why I just slept today &amp; did nothing else.</t>
+  </si>
+  <si>
+    <t>Today was the most descrnt day &amp; It was very soothing, No sunny day nice &amp; swift breeze.</t>
   </si>
 </sst>
 </file>
@@ -1494,27 +1497,51 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="18"/>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="20" t="str">
+    <row r="15" spans="1:14" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A15" s="18">
+        <v>46253</v>
+      </c>
+      <c r="B15" s="19">
+        <v>330</v>
+      </c>
+      <c r="C15" s="19">
+        <v>60</v>
+      </c>
+      <c r="D15" s="19">
+        <v>120</v>
+      </c>
+      <c r="E15" s="19">
+        <v>40</v>
+      </c>
+      <c r="F15" s="19">
+        <v>350</v>
+      </c>
+      <c r="G15" s="19">
+        <v>7</v>
+      </c>
+      <c r="H15" s="19">
+        <v>300</v>
+      </c>
+      <c r="I15" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="20" t="str">
+        <v>1200</v>
+      </c>
+      <c r="J15" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="22"/>
+        <v>240</v>
+      </c>
+      <c r="K15" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L15" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M15" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N15" s="22" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="16" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="18"/>

</xml_diff>

<commit_message>
Updated to 20th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="139" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{66EFFD25-626B-401C-9793-6B80229D6872}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20AA0EEE-65EB-466C-97D2-DA4E6E675FB3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -256,6 +256,9 @@
   </si>
   <si>
     <t>Today was the most descrnt day &amp; It was very soothing, No sunny day nice &amp; swift breeze.</t>
+  </si>
+  <si>
+    <t>Today there was some event in the hostel happened &amp; there were only 3 classes instead of 5 due to teacher's abscent</t>
   </si>
 </sst>
 </file>
@@ -1543,27 +1546,51 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="18"/>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
-      <c r="E16" s="19"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="20" t="str">
+    <row r="16" spans="1:14" ht="78" x14ac:dyDescent="0.3">
+      <c r="A16" s="18">
+        <v>46254</v>
+      </c>
+      <c r="B16" s="19">
+        <v>390</v>
+      </c>
+      <c r="C16" s="19">
+        <v>20</v>
+      </c>
+      <c r="D16" s="19">
+        <v>0</v>
+      </c>
+      <c r="E16" s="19">
+        <v>0</v>
+      </c>
+      <c r="F16" s="19">
+        <v>150</v>
+      </c>
+      <c r="G16" s="19">
+        <v>3</v>
+      </c>
+      <c r="H16" s="19">
+        <v>0</v>
+      </c>
+      <c r="I16" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="20" t="str">
+        <v>560</v>
+      </c>
+      <c r="J16" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="21"/>
-      <c r="L16" s="21"/>
-      <c r="M16" s="21"/>
-      <c r="N16" s="22"/>
+        <v>880</v>
+      </c>
+      <c r="K16" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="L16" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M16" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N16" s="22" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="17" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="18"/>

</xml_diff>

<commit_message>
Update for 21st August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20AA0EEE-65EB-466C-97D2-DA4E6E675FB3}"/>
+  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B63D1C77-BD07-41F1-8010-C08C43A0C206}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="75">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -259,6 +259,9 @@
   </si>
   <si>
     <t>Today there was some event in the hostel happened &amp; there were only 3 classes instead of 5 due to teacher's abscent</t>
+  </si>
+  <si>
+    <t>Today there was State close event due to which many classess were disrupted, &amp; class productivity was very low.</t>
   </si>
 </sst>
 </file>
@@ -1592,27 +1595,51 @@
         <v>73</v>
       </c>
     </row>
-    <row r="17" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="18"/>
-      <c r="B17" s="19"/>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="20" t="str">
+    <row r="17" spans="1:14" ht="78" x14ac:dyDescent="0.3">
+      <c r="A17" s="18">
+        <v>46255</v>
+      </c>
+      <c r="B17" s="19">
+        <v>420</v>
+      </c>
+      <c r="C17" s="19">
+        <v>28</v>
+      </c>
+      <c r="D17" s="19">
+        <v>120</v>
+      </c>
+      <c r="E17" s="19">
+        <v>50</v>
+      </c>
+      <c r="F17" s="19">
+        <v>100</v>
+      </c>
+      <c r="G17" s="19">
+        <v>2</v>
+      </c>
+      <c r="H17" s="19">
+        <v>400</v>
+      </c>
+      <c r="I17" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="20" t="str">
+        <v>1118</v>
+      </c>
+      <c r="J17" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="22"/>
+        <v>322</v>
+      </c>
+      <c r="K17" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L17" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="M17" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N17" s="22" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="18" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="18"/>

</xml_diff>

<commit_message>
Updated for 22nd August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="165" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B63D1C77-BD07-41F1-8010-C08C43A0C206}"/>
+  <xr:revisionPtr revIDLastSave="177" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E61A5497-712D-4EC6-87EC-757D7FEA1918}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="76">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -262,6 +262,9 @@
   </si>
   <si>
     <t>Today there was State close event due to which many classess were disrupted, &amp; class productivity was very low.</t>
+  </si>
+  <si>
+    <t>Today was the Holiday &amp; just a normal day, Nothing new happened.</t>
   </si>
 </sst>
 </file>
@@ -1641,27 +1644,51 @@
         <v>74</v>
       </c>
     </row>
-    <row r="18" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="18"/>
-      <c r="B18" s="19"/>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="20" t="str">
+    <row r="18" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A18" s="18">
+        <v>46256</v>
+      </c>
+      <c r="B18" s="19">
+        <v>420</v>
+      </c>
+      <c r="C18" s="19">
+        <v>10</v>
+      </c>
+      <c r="D18" s="19">
+        <v>190</v>
+      </c>
+      <c r="E18" s="19">
+        <v>45</v>
+      </c>
+      <c r="F18" s="19">
+        <v>0</v>
+      </c>
+      <c r="G18" s="19">
+        <v>0</v>
+      </c>
+      <c r="H18" s="19">
+        <v>0</v>
+      </c>
+      <c r="I18" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="20" t="str">
+        <v>665</v>
+      </c>
+      <c r="J18" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="21"/>
-      <c r="L18" s="21"/>
-      <c r="M18" s="21"/>
-      <c r="N18" s="22"/>
+        <v>775</v>
+      </c>
+      <c r="K18" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L18" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M18" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N18" s="22" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="19" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="18"/>

</xml_diff>

<commit_message>
Updated for 23rd August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="177" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E61A5497-712D-4EC6-87EC-757D7FEA1918}"/>
+  <xr:revisionPtr revIDLastSave="189" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAD1F671-9A78-44CB-98C3-71BBFB1D724C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -265,6 +265,9 @@
   </si>
   <si>
     <t>Today was the Holiday &amp; just a normal day, Nothing new happened.</t>
+  </si>
+  <si>
+    <t>Today I did some coding but before doing it I did write the code on the paper &amp; checked it manually by predicting the output.</t>
   </si>
 </sst>
 </file>
@@ -1690,27 +1693,51 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="18"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="20" t="str">
+    <row r="19" spans="1:14" ht="78" x14ac:dyDescent="0.3">
+      <c r="A19" s="18">
+        <v>46257</v>
+      </c>
+      <c r="B19" s="19">
+        <v>540</v>
+      </c>
+      <c r="C19" s="19">
+        <v>0</v>
+      </c>
+      <c r="D19" s="19">
+        <v>180</v>
+      </c>
+      <c r="E19" s="19">
+        <v>25</v>
+      </c>
+      <c r="F19" s="19">
+        <v>0</v>
+      </c>
+      <c r="G19" s="19">
+        <v>0</v>
+      </c>
+      <c r="H19" s="19">
+        <v>0</v>
+      </c>
+      <c r="I19" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="20" t="str">
+        <v>745</v>
+      </c>
+      <c r="J19" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="21"/>
-      <c r="N19" s="22"/>
+        <v>695</v>
+      </c>
+      <c r="K19" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L19" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M19" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N19" s="22" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="20" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="18"/>

</xml_diff>

<commit_message>
Updated for 24th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="189" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AAD1F671-9A78-44CB-98C3-71BBFB1D724C}"/>
+  <xr:revisionPtr revIDLastSave="202" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{845DD094-A631-4431-8BBA-1AA2D5694770}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -268,6 +268,9 @@
   </si>
   <si>
     <t>Today I did some coding but before doing it I did write the code on the paper &amp; checked it manually by predicting the output.</t>
+  </si>
+  <si>
+    <t>It was a nice day today, we got soe information about the C.A. which will happen next Monday</t>
   </si>
 </sst>
 </file>
@@ -1739,27 +1742,51 @@
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="18"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="20" t="str">
+    <row r="20" spans="1:14" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A20" s="18">
+        <v>46258</v>
+      </c>
+      <c r="B20" s="19">
+        <v>420</v>
+      </c>
+      <c r="C20" s="19">
+        <v>10</v>
+      </c>
+      <c r="D20" s="19">
+        <v>125</v>
+      </c>
+      <c r="E20" s="19">
+        <v>10</v>
+      </c>
+      <c r="F20" s="19">
+        <v>150</v>
+      </c>
+      <c r="G20" s="19">
+        <v>3</v>
+      </c>
+      <c r="H20" s="19">
+        <v>420</v>
+      </c>
+      <c r="I20" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="20" t="str">
+        <v>1135</v>
+      </c>
+      <c r="J20" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21"/>
-      <c r="M20" s="21"/>
-      <c r="N20" s="22"/>
+        <v>305</v>
+      </c>
+      <c r="K20" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L20" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="M20" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N20" s="22" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="18"/>

</xml_diff>

<commit_message>
Updated for 25th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="202" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{845DD094-A631-4431-8BBA-1AA2D5694770}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5B838E8-22EE-4EE5-9743-E42EA99C2859}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="79">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -271,6 +271,9 @@
   </si>
   <si>
     <t>It was a nice day today, we got soe information about the C.A. which will happen next Monday</t>
+  </si>
+  <si>
+    <t>Today we had The communication classes &amp; today was the start of the 3 DAY HELL WEEK. You will get to Know more tomorrow.</t>
   </si>
 </sst>
 </file>
@@ -1788,27 +1791,51 @@
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="18"/>
-      <c r="B21" s="19"/>
-      <c r="C21" s="19"/>
-      <c r="D21" s="19"/>
-      <c r="E21" s="19"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="20" t="str">
+    <row r="21" spans="1:14" ht="93.6" x14ac:dyDescent="0.3">
+      <c r="A21" s="18">
+        <v>46259</v>
+      </c>
+      <c r="B21" s="19">
+        <v>390</v>
+      </c>
+      <c r="C21" s="19">
+        <v>25</v>
+      </c>
+      <c r="D21" s="19">
+        <v>145</v>
+      </c>
+      <c r="E21" s="19">
+        <v>0</v>
+      </c>
+      <c r="F21" s="19">
+        <v>300</v>
+      </c>
+      <c r="G21" s="19">
+        <v>6</v>
+      </c>
+      <c r="H21" s="19">
+        <v>300</v>
+      </c>
+      <c r="I21" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="20" t="str">
+        <v>1160</v>
+      </c>
+      <c r="J21" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="22"/>
+        <v>280</v>
+      </c>
+      <c r="K21" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="L21" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M21" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N21" s="22" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="22" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="18"/>

</xml_diff>

<commit_message>
Updated for 26th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B5B838E8-22EE-4EE5-9743-E42EA99C2859}"/>
+  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{856E8C21-A870-462F-85DE-B2CCF47D7244}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="80">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -274,6 +274,9 @@
   </si>
   <si>
     <t>Today we had The communication classes &amp; today was the start of the 3 DAY HELL WEEK. You will get to Know more tomorrow.</t>
+  </si>
+  <si>
+    <t>Today there were 8 classes &amp; we did some project questions.</t>
   </si>
 </sst>
 </file>
@@ -1837,27 +1840,51 @@
         <v>78</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="18"/>
-      <c r="B22" s="19"/>
-      <c r="C22" s="19"/>
-      <c r="D22" s="19"/>
-      <c r="E22" s="19"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="20" t="str">
+    <row r="22" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A22" s="18">
+        <v>46260</v>
+      </c>
+      <c r="B22" s="19">
+        <v>480</v>
+      </c>
+      <c r="C22" s="19">
+        <v>32</v>
+      </c>
+      <c r="D22" s="19">
+        <v>120</v>
+      </c>
+      <c r="E22" s="19">
+        <v>20</v>
+      </c>
+      <c r="F22" s="19">
+        <v>400</v>
+      </c>
+      <c r="G22" s="19">
+        <v>8</v>
+      </c>
+      <c r="H22" s="19">
+        <v>200</v>
+      </c>
+      <c r="I22" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="20" t="str">
+        <v>1252</v>
+      </c>
+      <c r="J22" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="21"/>
-      <c r="L22" s="21"/>
-      <c r="M22" s="21"/>
-      <c r="N22" s="22"/>
+        <v>188</v>
+      </c>
+      <c r="K22" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="L22" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M22" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N22" s="22" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="23" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="18"/>

</xml_diff>

<commit_message>
Updated for 27th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="226" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{856E8C21-A870-462F-85DE-B2CCF47D7244}"/>
+  <xr:revisionPtr revIDLastSave="239" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CFCD8C7-85FE-44FE-B552-869615F3E35E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="81">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -277,6 +277,9 @@
   </si>
   <si>
     <t>Today there were 8 classes &amp; we did some project questions.</t>
+  </si>
+  <si>
+    <t>Today I had shoping for Tomorrow's Rakshabandhan Festival.</t>
   </si>
 </sst>
 </file>
@@ -1886,27 +1889,51 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="18"/>
-      <c r="B23" s="19"/>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="20" t="str">
+    <row r="23" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A23" s="18">
+        <v>46261</v>
+      </c>
+      <c r="B23" s="19">
+        <v>450</v>
+      </c>
+      <c r="C23" s="19">
+        <v>45</v>
+      </c>
+      <c r="D23" s="19">
+        <v>124</v>
+      </c>
+      <c r="E23" s="19">
+        <v>44</v>
+      </c>
+      <c r="F23" s="19">
+        <v>250</v>
+      </c>
+      <c r="G23" s="19">
+        <v>5</v>
+      </c>
+      <c r="H23" s="19">
+        <v>100</v>
+      </c>
+      <c r="I23" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="20" t="str">
+        <v>1013</v>
+      </c>
+      <c r="J23" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="21"/>
-      <c r="L23" s="21"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="22"/>
+        <v>427</v>
+      </c>
+      <c r="K23" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L23" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M23" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N23" s="22" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="18"/>

</xml_diff>

<commit_message>
Updated for 29th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="239" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CFCD8C7-85FE-44FE-B552-869615F3E35E}"/>
+  <xr:revisionPtr revIDLastSave="264" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67C51504-9A8F-41A3-87C4-52E39C83F45E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="83">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -280,6 +280,12 @@
   </si>
   <si>
     <t>Today I had shoping for Tomorrow's Rakshabandhan Festival.</t>
+  </si>
+  <si>
+    <t>Today one class got cancelled &amp; due to that we have a new makeup class tomorrow.</t>
+  </si>
+  <si>
+    <t>Today I take leave to purchase the Dresses for the CA that is going to happen in the next week.</t>
   </si>
 </sst>
 </file>
@@ -1935,49 +1941,97 @@
         <v>80</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="18"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="20" t="str">
+    <row r="24" spans="1:14" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A24" s="18">
+        <v>46262</v>
+      </c>
+      <c r="B24" s="19">
+        <v>420</v>
+      </c>
+      <c r="C24" s="19">
+        <v>20</v>
+      </c>
+      <c r="D24" s="19">
+        <v>0</v>
+      </c>
+      <c r="E24" s="19">
+        <v>0</v>
+      </c>
+      <c r="F24" s="19">
+        <v>200</v>
+      </c>
+      <c r="G24" s="19">
+        <v>4</v>
+      </c>
+      <c r="H24" s="19">
+        <v>0</v>
+      </c>
+      <c r="I24" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="20" t="str">
+        <v>640</v>
+      </c>
+      <c r="J24" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K24" s="21"/>
-      <c r="L24" s="21"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="22"/>
-    </row>
-    <row r="25" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="18"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="20" t="str">
+        <v>800</v>
+      </c>
+      <c r="K24" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L24" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M24" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N24" s="22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A25" s="18">
+        <v>46263</v>
+      </c>
+      <c r="B25" s="19">
+        <v>360</v>
+      </c>
+      <c r="C25" s="19">
+        <v>35</v>
+      </c>
+      <c r="D25" s="19">
+        <v>0</v>
+      </c>
+      <c r="E25" s="19">
+        <v>0</v>
+      </c>
+      <c r="F25" s="19">
+        <v>65</v>
+      </c>
+      <c r="G25" s="19">
+        <v>1</v>
+      </c>
+      <c r="H25" s="19">
+        <v>500</v>
+      </c>
+      <c r="I25" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="20" t="str">
+        <v>960</v>
+      </c>
+      <c r="J25" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K25" s="21"/>
-      <c r="L25" s="21"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="22"/>
+        <v>480</v>
+      </c>
+      <c r="K25" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L25" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M25" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N25" s="22" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="26" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="18"/>

</xml_diff>

<commit_message>
Update for 30th August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="264" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67C51504-9A8F-41A3-87C4-52E39C83F45E}"/>
+  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4F261DE-19A0-4EA0-B610-2B764FD43A4E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>Today I take leave to purchase the Dresses for the CA that is going to happen in the next week.</t>
+  </si>
+  <si>
+    <t>Today I just Practiced for the upcoming CA</t>
   </si>
 </sst>
 </file>
@@ -2033,27 +2036,51 @@
         <v>82</v>
       </c>
     </row>
-    <row r="26" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="18"/>
-      <c r="B26" s="19"/>
-      <c r="C26" s="19"/>
-      <c r="D26" s="19"/>
-      <c r="E26" s="19"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="20" t="str">
+    <row r="26" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A26" s="18">
+        <v>46264</v>
+      </c>
+      <c r="B26" s="19">
+        <v>420</v>
+      </c>
+      <c r="C26" s="19">
+        <v>0</v>
+      </c>
+      <c r="D26" s="19">
+        <v>60</v>
+      </c>
+      <c r="E26" s="19">
+        <v>0</v>
+      </c>
+      <c r="F26" s="19">
+        <v>0</v>
+      </c>
+      <c r="G26" s="19">
+        <v>0</v>
+      </c>
+      <c r="H26" s="19">
+        <v>300</v>
+      </c>
+      <c r="I26" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="20" t="str">
+        <v>780</v>
+      </c>
+      <c r="J26" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K26" s="21"/>
-      <c r="L26" s="21"/>
-      <c r="M26" s="21"/>
-      <c r="N26" s="22"/>
+        <v>660</v>
+      </c>
+      <c r="K26" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L26" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M26" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N26" s="22" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="27" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="18"/>

</xml_diff>

<commit_message>
Updated for 31st August
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4F261DE-19A0-4EA0-B610-2B764FD43A4E}"/>
+  <xr:revisionPtr revIDLastSave="289" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04682562-8392-4011-AA7F-46DB94497D7F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="85">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -289,6 +289,9 @@
   </si>
   <si>
     <t>Today I just Practiced for the upcoming CA</t>
+  </si>
+  <si>
+    <t>Today some classes were canceled due to the career counselling presentation.</t>
   </si>
 </sst>
 </file>
@@ -2082,27 +2085,51 @@
         <v>83</v>
       </c>
     </row>
-    <row r="27" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="18"/>
-      <c r="B27" s="19"/>
-      <c r="C27" s="19"/>
-      <c r="D27" s="19"/>
-      <c r="E27" s="19"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="20" t="str">
+    <row r="27" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A27" s="18">
+        <v>46265</v>
+      </c>
+      <c r="B27" s="19">
+        <v>460</v>
+      </c>
+      <c r="C27" s="19">
+        <v>30</v>
+      </c>
+      <c r="D27" s="19">
+        <v>140</v>
+      </c>
+      <c r="E27" s="19">
+        <v>35</v>
+      </c>
+      <c r="F27" s="19">
+        <v>50</v>
+      </c>
+      <c r="G27" s="19">
+        <v>1</v>
+      </c>
+      <c r="H27" s="19">
+        <v>540</v>
+      </c>
+      <c r="I27" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="20" t="str">
+        <v>1255</v>
+      </c>
+      <c r="J27" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K27" s="21"/>
-      <c r="L27" s="21"/>
-      <c r="M27" s="21"/>
-      <c r="N27" s="22"/>
+        <v>185</v>
+      </c>
+      <c r="K27" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L27" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="M27" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N27" s="22" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="28" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="18"/>

</xml_diff>

<commit_message>
Updated for 1st September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="289" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{04682562-8392-4011-AA7F-46DB94497D7F}"/>
+  <xr:revisionPtr revIDLastSave="301" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F4FAE54-C635-4699-B360-6D14BDC51D69}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -292,6 +292,9 @@
   </si>
   <si>
     <t>Today some classes were canceled due to the career counselling presentation.</t>
+  </si>
+  <si>
+    <t>Today I read for tomorrow's CA, &amp; it will in the first class.</t>
   </si>
 </sst>
 </file>
@@ -2131,27 +2134,51 @@
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="18"/>
-      <c r="B28" s="19"/>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="20" t="str">
+    <row r="28" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A28" s="18">
+        <v>46266</v>
+      </c>
+      <c r="B28" s="19">
+        <v>390</v>
+      </c>
+      <c r="C28" s="19">
+        <v>30</v>
+      </c>
+      <c r="D28" s="19">
+        <v>120</v>
+      </c>
+      <c r="E28" s="19">
+        <v>0</v>
+      </c>
+      <c r="F28" s="19">
+        <v>300</v>
+      </c>
+      <c r="G28" s="19">
+        <v>6</v>
+      </c>
+      <c r="H28" s="19">
+        <v>0</v>
+      </c>
+      <c r="I28" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="20" t="str">
+        <v>840</v>
+      </c>
+      <c r="J28" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="21"/>
-      <c r="L28" s="21"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="22"/>
+        <v>600</v>
+      </c>
+      <c r="K28" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L28" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M28" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N28" s="22" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="29" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="18"/>

</xml_diff>

<commit_message>
Updated for 2nd September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="301" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9F4FAE54-C635-4699-B360-6D14BDC51D69}"/>
+  <xr:revisionPtr revIDLastSave="313" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{844EB9A1-00E8-40C2-8679-DD4552C73276}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="87">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -295,6 +295,9 @@
   </si>
   <si>
     <t>Today I read for tomorrow's CA, &amp; it will in the first class.</t>
+  </si>
+  <si>
+    <t>Today I ahd CA in Communication &amp; I got to knoe the upcoming CA in the next week.</t>
   </si>
 </sst>
 </file>
@@ -2180,27 +2183,51 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="18"/>
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="20" t="str">
+    <row r="29" spans="1:14" ht="62.4" x14ac:dyDescent="0.3">
+      <c r="A29" s="18">
+        <v>46267</v>
+      </c>
+      <c r="B29" s="19">
+        <v>390</v>
+      </c>
+      <c r="C29" s="19">
+        <v>49</v>
+      </c>
+      <c r="D29" s="19">
+        <v>65</v>
+      </c>
+      <c r="E29" s="19">
+        <v>20</v>
+      </c>
+      <c r="F29" s="19">
+        <v>400</v>
+      </c>
+      <c r="G29" s="19">
+        <v>8</v>
+      </c>
+      <c r="H29" s="19">
+        <v>300</v>
+      </c>
+      <c r="I29" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="20" t="str">
+        <v>1224</v>
+      </c>
+      <c r="J29" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K29" s="21"/>
-      <c r="L29" s="21"/>
-      <c r="M29" s="21"/>
-      <c r="N29" s="22"/>
+        <v>216</v>
+      </c>
+      <c r="K29" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L29" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="M29" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="N29" s="22" t="s">
+        <v>86</v>
+      </c>
     </row>
     <row r="30" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="18"/>

</xml_diff>

<commit_message>
Updated for 3rd September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="313" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{844EB9A1-00E8-40C2-8679-DD4552C73276}"/>
+  <xr:revisionPtr revIDLastSave="325" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7A9D1D3-6280-42FB-91BE-EBCA271D44D0}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="88">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -298,6 +298,9 @@
   </si>
   <si>
     <t>Today I ahd CA in Communication &amp; I got to knoe the upcoming CA in the next week.</t>
+  </si>
+  <si>
+    <t>Today we Decided to make a Project Group with atleast 5 members.</t>
   </si>
 </sst>
 </file>
@@ -2229,27 +2232,51 @@
         <v>86</v>
       </c>
     </row>
-    <row r="30" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="18"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="20" t="str">
+    <row r="30" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A30" s="18">
+        <v>46268</v>
+      </c>
+      <c r="B30" s="19">
+        <v>360</v>
+      </c>
+      <c r="C30" s="19">
+        <v>50</v>
+      </c>
+      <c r="D30" s="19">
+        <v>120</v>
+      </c>
+      <c r="E30" s="19">
+        <v>20</v>
+      </c>
+      <c r="F30" s="19">
+        <v>150</v>
+      </c>
+      <c r="G30" s="19">
+        <v>3</v>
+      </c>
+      <c r="H30" s="19">
+        <v>200</v>
+      </c>
+      <c r="I30" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="20" t="str">
+        <v>900</v>
+      </c>
+      <c r="J30" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K30" s="21"/>
-      <c r="L30" s="21"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="22"/>
+        <v>540</v>
+      </c>
+      <c r="K30" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="L30" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M30" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="N30" s="22" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="31" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="18"/>

</xml_diff>

<commit_message>
Updated for 4th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="325" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D7A9D1D3-6280-42FB-91BE-EBCA271D44D0}"/>
+  <xr:revisionPtr revIDLastSave="339" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B2061E3-B245-4837-B61D-0E60085CF03F}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="89">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -301,6 +301,9 @@
   </si>
   <si>
     <t>Today we Decided to make a Project Group with atleast 5 members.</t>
+  </si>
+  <si>
+    <t>Today we did some Analytical Questions &amp; did some coding.</t>
   </si>
 </sst>
 </file>
@@ -2278,27 +2281,51 @@
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="18"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="19"/>
-      <c r="D31" s="19"/>
-      <c r="E31" s="19"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="20" t="str">
+    <row r="31" spans="1:14" ht="46.8" x14ac:dyDescent="0.3">
+      <c r="A31" s="18">
+        <v>46269</v>
+      </c>
+      <c r="B31" s="19">
+        <v>300</v>
+      </c>
+      <c r="C31" s="19">
+        <v>45</v>
+      </c>
+      <c r="D31" s="19">
+        <v>78</v>
+      </c>
+      <c r="E31" s="19">
+        <v>36</v>
+      </c>
+      <c r="F31" s="19">
+        <v>150</v>
+      </c>
+      <c r="G31" s="19">
+        <v>3</v>
+      </c>
+      <c r="H31" s="19">
+        <v>0</v>
+      </c>
+      <c r="I31" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J31" s="20" t="str">
+        <v>609</v>
+      </c>
+      <c r="J31" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K31" s="21"/>
-      <c r="L31" s="21"/>
-      <c r="M31" s="21"/>
-      <c r="N31" s="22"/>
+        <v>831</v>
+      </c>
+      <c r="K31" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L31" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M31" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N31" s="22" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="32" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="18"/>

</xml_diff>

<commit_message>
Updated for 5th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="339" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7B2061E3-B245-4837-B61D-0E60085CF03F}"/>
+  <xr:revisionPtr revIDLastSave="352" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D8D010A-E6BA-405E-A5D2-E97461E036BE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="90">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -304,6 +304,9 @@
   </si>
   <si>
     <t>Today we did some Analytical Questions &amp; did some coding.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Today I read some notes of DBMS. </t>
   </si>
 </sst>
 </file>
@@ -2327,27 +2330,51 @@
         <v>88</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="18"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="19"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="19"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="20" t="str">
+    <row r="32" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A32" s="18">
+        <v>46270</v>
+      </c>
+      <c r="B32" s="19">
+        <v>375</v>
+      </c>
+      <c r="C32" s="19">
+        <v>25</v>
+      </c>
+      <c r="D32" s="19">
+        <v>120</v>
+      </c>
+      <c r="E32" s="19">
+        <v>0</v>
+      </c>
+      <c r="F32" s="19">
+        <v>0</v>
+      </c>
+      <c r="G32" s="19">
+        <v>0</v>
+      </c>
+      <c r="H32" s="19">
+        <v>0</v>
+      </c>
+      <c r="I32" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J32" s="20" t="str">
+        <v>520</v>
+      </c>
+      <c r="J32" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="22"/>
+        <v>920</v>
+      </c>
+      <c r="K32" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="L32" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="M32" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N32" s="22" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="33" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="18"/>

</xml_diff>

<commit_message>
Updated for 6th September
</commit_message>
<xml_diff>
--- a/12601870.xlsx
+++ b/12601870.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/370a177e9e66eb08/Documents/GitHub/Daily-Activity-tracker-CAP776-Python/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="352" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5D8D010A-E6BA-405E-A5D2-E97461E036BE}"/>
+  <xr:revisionPtr revIDLastSave="365" documentId="13_ncr:1_{1A11B410-6228-4EFB-ADF5-2519D16142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6071D77-6F8B-43C2-8862-E0F42BBAFBB5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="91">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -307,6 +307,9 @@
   </si>
   <si>
     <t xml:space="preserve">Today I read some notes of DBMS. </t>
+  </si>
+  <si>
+    <t>Today I started prepairing for the CA</t>
   </si>
 </sst>
 </file>
@@ -2376,27 +2379,51 @@
         <v>89</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="18"/>
-      <c r="B33" s="19"/>
-      <c r="C33" s="19"/>
-      <c r="D33" s="19"/>
-      <c r="E33" s="19"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="20" t="str">
+    <row r="33" spans="1:14" ht="31.2" x14ac:dyDescent="0.3">
+      <c r="A33" s="18">
+        <v>46271</v>
+      </c>
+      <c r="B33" s="19">
+        <v>540</v>
+      </c>
+      <c r="C33" s="19">
+        <v>35</v>
+      </c>
+      <c r="D33" s="19">
+        <v>90</v>
+      </c>
+      <c r="E33" s="19">
+        <v>25</v>
+      </c>
+      <c r="F33" s="19">
+        <v>0</v>
+      </c>
+      <c r="G33" s="19">
+        <v>0</v>
+      </c>
+      <c r="H33" s="19">
+        <v>0</v>
+      </c>
+      <c r="I33" s="20">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="20" t="str">
+        <v>690</v>
+      </c>
+      <c r="J33" s="20">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="21"/>
-      <c r="L33" s="21"/>
-      <c r="M33" s="21"/>
-      <c r="N33" s="22"/>
+        <v>750</v>
+      </c>
+      <c r="K33" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="L33" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="M33" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="N33" s="22" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="34" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="18"/>

</xml_diff>